<commit_message>
데이터 업데이트 2026-05-26 (벌크 6691개, MAE 11.80%)
</commit_message>
<xml_diff>
--- a/data/disposal.xlsx
+++ b/data/disposal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cosmaxdt-my.sharepoint.com/personal/djlee_cosmax_com/Documents/바탕 화면/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="131" documentId="8_{130E5389-1375-4C82-BE1D-2D037779CF4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91C0208D-646A-4777-B9FB-AA5C733632BE}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{130E5389-1375-4C82-BE1D-2D037779CF4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A81B6BFD-70B9-4E0E-9C9D-D23061C84D92}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{156CA689-9E30-4938-99C3-2C7A464D90AA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1569" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="853">
   <si>
     <t>생산오더</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2852,6 +2852,282 @@
   </si>
   <si>
     <t>3DZK00089190</t>
+  </si>
+  <si>
+    <t>3IWD00432171</t>
+  </si>
+  <si>
+    <t>33AC01066120</t>
+  </si>
+  <si>
+    <t>3IWD00404150</t>
+  </si>
+  <si>
+    <t>3IWD00433140</t>
+  </si>
+  <si>
+    <t>3IWD00433130</t>
+  </si>
+  <si>
+    <t>3IWD00432161</t>
+  </si>
+  <si>
+    <t>3CLO13069200</t>
+  </si>
+  <si>
+    <t>33AC01067120</t>
+  </si>
+  <si>
+    <t>3IWD00404101</t>
+  </si>
+  <si>
+    <t>3IWD00404120</t>
+  </si>
+  <si>
+    <t>3CLO13069150</t>
+  </si>
+  <si>
+    <t>3MEM08597110</t>
+  </si>
+  <si>
+    <t>3DZK00024170</t>
+  </si>
+  <si>
+    <t>3DZK00024121</t>
+  </si>
+  <si>
+    <t>3CLO13069210</t>
+  </si>
+  <si>
+    <t>3IWD00432120</t>
+  </si>
+  <si>
+    <t>3DZK00024180</t>
+  </si>
+  <si>
+    <t>3DZK00024140</t>
+  </si>
+  <si>
+    <t>3DZK00024131</t>
+  </si>
+  <si>
+    <t>3DZK00024190</t>
+  </si>
+  <si>
+    <t>3DZK00024160</t>
+  </si>
+  <si>
+    <t>3CLO13982160</t>
+  </si>
+  <si>
+    <t>3IAN10370150</t>
+  </si>
+  <si>
+    <t>3IAN00092120</t>
+  </si>
+  <si>
+    <t>3IAN10370160</t>
+  </si>
+  <si>
+    <t>3CLO13009130</t>
+  </si>
+  <si>
+    <t>3IAN00096150</t>
+  </si>
+  <si>
+    <t>3IAN00092140</t>
+  </si>
+  <si>
+    <t>3DZK00504190</t>
+  </si>
+  <si>
+    <t>3IAN10370120</t>
+  </si>
+  <si>
+    <t>3IAN10370140</t>
+  </si>
+  <si>
+    <t>3IAN00092150</t>
+  </si>
+  <si>
+    <t>3CLO13069120</t>
+  </si>
+  <si>
+    <t>3IWD00331110</t>
+  </si>
+  <si>
+    <t>3CLO13232220</t>
+  </si>
+  <si>
+    <t>3IAN10219150</t>
+  </si>
+  <si>
+    <t>3MEM08595110</t>
+  </si>
+  <si>
+    <t>3IWD00433170</t>
+  </si>
+  <si>
+    <t>3MEM00771120</t>
+  </si>
+  <si>
+    <t>3IAN10371110</t>
+  </si>
+  <si>
+    <t>3IAN10370130</t>
+  </si>
+  <si>
+    <t>3CLO14002130</t>
+  </si>
+  <si>
+    <t>3ENP00739110</t>
+  </si>
+  <si>
+    <t>3CLO13973130</t>
+  </si>
+  <si>
+    <t>3IAN10370110</t>
+  </si>
+  <si>
+    <t>3CLO13973110</t>
+  </si>
+  <si>
+    <t>3CLO13973140</t>
+  </si>
+  <si>
+    <t>3IAN10378110</t>
+  </si>
+  <si>
+    <t>3IAN00020111</t>
+  </si>
+  <si>
+    <t>3NRP01710110</t>
+  </si>
+  <si>
+    <t>3CLO13750140</t>
+  </si>
+  <si>
+    <t>3NRP01687119</t>
+  </si>
+  <si>
+    <t>3MSA00033110</t>
+  </si>
+  <si>
+    <t>3MSA00033140</t>
+  </si>
+  <si>
+    <t>3MEM00631152</t>
+  </si>
+  <si>
+    <t>3DZK00574140</t>
+  </si>
+  <si>
+    <t>3COS05997110</t>
+  </si>
+  <si>
+    <t>3MEM00631142</t>
+  </si>
+  <si>
+    <t>3COS81834110</t>
+  </si>
+  <si>
+    <t>3COS81833110</t>
+  </si>
+  <si>
+    <t>3COS81832110</t>
+  </si>
+  <si>
+    <t>3COS05994110</t>
+  </si>
+  <si>
+    <t>3DZK00089130</t>
+  </si>
+  <si>
+    <t>3MEM00631112</t>
+  </si>
+  <si>
+    <t>3COS05996110</t>
+  </si>
+  <si>
+    <t>3NRP01577220</t>
+  </si>
+  <si>
+    <t>3OLV11236135</t>
+  </si>
+  <si>
+    <t>3NRP01577230</t>
+  </si>
+  <si>
+    <t>3LOJ01284110</t>
+  </si>
+  <si>
+    <t>3NRP01577240</t>
+  </si>
+  <si>
+    <t>3ENP00738160</t>
+  </si>
+  <si>
+    <t>3NRP01709220</t>
+  </si>
+  <si>
+    <t>3MEM08540120</t>
+  </si>
+  <si>
+    <t>3MEM00567170</t>
+  </si>
+  <si>
+    <t>3ENP00738130</t>
+  </si>
+  <si>
+    <t>3LOJ01287110</t>
+  </si>
+  <si>
+    <t>3MEM08540130</t>
+  </si>
+  <si>
+    <t>3MEM00567140</t>
+  </si>
+  <si>
+    <t>3NRP01709230</t>
+  </si>
+  <si>
+    <t>3DZK00024150</t>
+  </si>
+  <si>
+    <t>3MEM00678112</t>
+  </si>
+  <si>
+    <t>3IWD00480110</t>
+  </si>
+  <si>
+    <t>3ENP00646111</t>
+  </si>
+  <si>
+    <t>3IWD00482110</t>
+  </si>
+  <si>
+    <t>3MEM00567110</t>
+  </si>
+  <si>
+    <t>3CLO13188170</t>
+  </si>
+  <si>
+    <t>3CLO13188171</t>
+  </si>
+  <si>
+    <t>3ENP00646121</t>
+  </si>
+  <si>
+    <t>3MEM00567120</t>
+  </si>
+  <si>
+    <t>3ENP00646131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3MEM00567130	</t>
+  </si>
+  <si>
+    <t>3MEM00567160</t>
   </si>
 </sst>
 </file>
@@ -3307,7 +3583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D5B24D8-C2AF-482A-9CC6-491ED0721327}">
-  <dimension ref="A1:F290"/>
+  <dimension ref="A1:F329"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" style="3" bestFit="1" customWidth="1"/>
@@ -8251,10 +8527,673 @@
         <v>46157</v>
       </c>
     </row>
+    <row r="291" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A291" s="3">
+        <v>503801398</v>
+      </c>
+      <c r="B291" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="C291" s="5">
+        <v>2100</v>
+      </c>
+      <c r="D291" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E291" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A292" s="3">
+        <v>503808145</v>
+      </c>
+      <c r="B292" s="3" t="s">
+        <v>816</v>
+      </c>
+      <c r="C292" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D292" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E292" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A293" s="3">
+        <v>503803591</v>
+      </c>
+      <c r="B293" s="3" t="s">
+        <v>817</v>
+      </c>
+      <c r="C293" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D293" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E293" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="294" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A294" s="3">
+        <v>503801397</v>
+      </c>
+      <c r="B294" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="C294" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D294" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E294" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="295" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A295" s="3">
+        <v>503784914</v>
+      </c>
+      <c r="B295" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="C295" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D295" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E295" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A296" s="3">
+        <v>503784914</v>
+      </c>
+      <c r="B296" s="3" t="s">
+        <v>820</v>
+      </c>
+      <c r="C296" s="5">
+        <v>500</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E296" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="297" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A297" s="3">
+        <v>503784914</v>
+      </c>
+      <c r="B297" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="C297" s="5">
+        <v>1000</v>
+      </c>
+      <c r="D297" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E297" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A298" s="3">
+        <v>503803588</v>
+      </c>
+      <c r="B298" s="3" t="s">
+        <v>822</v>
+      </c>
+      <c r="C298" s="5">
+        <v>500</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E298" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="299" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A299" s="3">
+        <v>503797692</v>
+      </c>
+      <c r="B299" s="3" t="s">
+        <v>823</v>
+      </c>
+      <c r="C299" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D299" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E299" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="300" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A300" s="3">
+        <v>503806323</v>
+      </c>
+      <c r="B300" s="3" t="s">
+        <v>824</v>
+      </c>
+      <c r="C300" s="5">
+        <v>2100</v>
+      </c>
+      <c r="D300" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E300" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="301" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A301" s="3">
+        <v>503803590</v>
+      </c>
+      <c r="B301" s="3" t="s">
+        <v>825</v>
+      </c>
+      <c r="C301" s="5">
+        <v>800</v>
+      </c>
+      <c r="D301" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E301" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="302" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A302" s="3">
+        <v>503806532</v>
+      </c>
+      <c r="B302" s="3" t="s">
+        <v>826</v>
+      </c>
+      <c r="C302" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D302" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E302" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="303" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A303" s="3">
+        <v>503801464</v>
+      </c>
+      <c r="B303" s="3" t="s">
+        <v>827</v>
+      </c>
+      <c r="C303" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D303" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E303" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="304" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A304" s="3">
+        <v>503806533</v>
+      </c>
+      <c r="B304" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="C304" s="5">
+        <v>2200</v>
+      </c>
+      <c r="D304" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E304" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="305" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A305" s="3">
+        <v>503808973</v>
+      </c>
+      <c r="B305" s="3" t="s">
+        <v>829</v>
+      </c>
+      <c r="C305" s="5">
+        <v>500</v>
+      </c>
+      <c r="D305" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E305" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="306" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A306" s="3">
+        <v>503806534</v>
+      </c>
+      <c r="B306" s="3" t="s">
+        <v>830</v>
+      </c>
+      <c r="C306" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D306" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E306" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="307" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A307" s="3">
+        <v>503809547</v>
+      </c>
+      <c r="B307" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="C307" s="5">
+        <v>1400</v>
+      </c>
+      <c r="D307" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E307" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="308" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A308" s="3">
+        <v>503807902</v>
+      </c>
+      <c r="B308" s="3" t="s">
+        <v>832</v>
+      </c>
+      <c r="C308" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D308" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E308" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="309" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A309" s="3">
+        <v>503814222</v>
+      </c>
+      <c r="B309" s="3" t="s">
+        <v>833</v>
+      </c>
+      <c r="C309" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D309" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E309" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="310" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A310" s="3">
+        <v>503812037</v>
+      </c>
+      <c r="B310" s="3" t="s">
+        <v>834</v>
+      </c>
+      <c r="C310" s="5">
+        <v>500</v>
+      </c>
+      <c r="D310" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E310" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="311" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A311" s="3">
+        <v>503809546</v>
+      </c>
+      <c r="B311" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="C311" s="5">
+        <v>1800</v>
+      </c>
+      <c r="D311" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E311" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="312" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A312" s="3">
+        <v>503812086</v>
+      </c>
+      <c r="B312" s="3" t="s">
+        <v>836</v>
+      </c>
+      <c r="C312" s="5">
+        <v>300</v>
+      </c>
+      <c r="D312" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E312" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="313" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A313" s="3">
+        <v>503814363</v>
+      </c>
+      <c r="B313" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="C313" s="5">
+        <v>2200</v>
+      </c>
+      <c r="D313" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E313" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="314" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A314" s="3">
+        <v>503812035</v>
+      </c>
+      <c r="B314" s="3" t="s">
+        <v>838</v>
+      </c>
+      <c r="C314" s="5">
+        <v>200</v>
+      </c>
+      <c r="D314" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E314" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="315" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A315" s="3">
+        <v>503808083</v>
+      </c>
+      <c r="B315" s="3" t="s">
+        <v>839</v>
+      </c>
+      <c r="C315" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D315" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E315" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="316" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A316" s="3">
+        <v>503809605</v>
+      </c>
+      <c r="B316" s="3" t="s">
+        <v>840</v>
+      </c>
+      <c r="C316" s="5">
+        <v>2600</v>
+      </c>
+      <c r="D316" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E316" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="317" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A317" s="3">
+        <v>503814364</v>
+      </c>
+      <c r="B317" s="3" t="s">
+        <v>841</v>
+      </c>
+      <c r="C317" s="5">
+        <v>500</v>
+      </c>
+      <c r="D317" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E317" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="318" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A318" s="3">
+        <v>503809052</v>
+      </c>
+      <c r="B318" s="3" t="s">
+        <v>842</v>
+      </c>
+      <c r="C318" s="5">
+        <v>300</v>
+      </c>
+      <c r="D318" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E318" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="319" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A319" s="3">
+        <v>503812042</v>
+      </c>
+      <c r="B319" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="C319" s="5">
+        <v>1900</v>
+      </c>
+      <c r="D319" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E319" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="320" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A320" s="3">
+        <v>503813538</v>
+      </c>
+      <c r="B320" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="C320" s="5">
+        <v>1600</v>
+      </c>
+      <c r="D320" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E320" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="321" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A321" s="3">
+        <v>503808977</v>
+      </c>
+      <c r="B321" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="C321" s="5">
+        <v>700</v>
+      </c>
+      <c r="D321" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E321" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="322" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A322" s="3">
+        <v>503812032</v>
+      </c>
+      <c r="B322" s="3" t="s">
+        <v>845</v>
+      </c>
+      <c r="C322" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D322" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E322" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="323" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A323" s="3">
+        <v>503809103</v>
+      </c>
+      <c r="B323" s="3" t="s">
+        <v>846</v>
+      </c>
+      <c r="C323" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D323" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E323" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="324" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A324" s="3">
+        <v>503809103</v>
+      </c>
+      <c r="B324" s="3" t="s">
+        <v>847</v>
+      </c>
+      <c r="C324" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D324" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E324" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="325" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A325" s="3">
+        <v>503812083</v>
+      </c>
+      <c r="B325" s="3" t="s">
+        <v>848</v>
+      </c>
+      <c r="C325" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D325" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E325" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="326" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A326" s="3">
+        <v>503812033</v>
+      </c>
+      <c r="B326" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="C326" s="5">
+        <v>1600</v>
+      </c>
+      <c r="D326" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E326" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="327" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A327" s="3">
+        <v>503812084</v>
+      </c>
+      <c r="B327" s="3" t="s">
+        <v>850</v>
+      </c>
+      <c r="C327" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D327" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E327" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="328" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A328" s="3">
+        <v>503812034</v>
+      </c>
+      <c r="B328" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="C328" s="5">
+        <v>2200</v>
+      </c>
+      <c r="D328" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E328" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="329" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A329" s="3">
+        <v>503812036</v>
+      </c>
+      <c r="B329" s="3" t="s">
+        <v>852</v>
+      </c>
+      <c r="C329" s="5">
+        <v>1800</v>
+      </c>
+      <c r="D329" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E329" s="6">
+        <v>46164</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F290" xr:uid="{4D5B24D8-C2AF-482A-9CC6-491ED0721327}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F290">
-      <sortCondition ref="E1:E135"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F329">
+      <sortCondition ref="E1:E290"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -8264,7 +9203,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2F62A61-38E3-43AD-974B-FDA325720BCC}">
-  <dimension ref="A1:F490"/>
+  <dimension ref="A1:F545"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" style="3" bestFit="1" customWidth="1"/>
@@ -16612,10 +17551,945 @@
         <v>46157</v>
       </c>
     </row>
+    <row r="491" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A491" s="3">
+        <v>503801285</v>
+      </c>
+      <c r="B491" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="C491" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D491" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E491" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="492" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A492" s="3">
+        <v>503800791</v>
+      </c>
+      <c r="B492" s="3" t="s">
+        <v>762</v>
+      </c>
+      <c r="C492" s="5">
+        <v>1100</v>
+      </c>
+      <c r="D492" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E492" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="493" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A493" s="3">
+        <v>503801294</v>
+      </c>
+      <c r="B493" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="C493" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D493" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E493" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="494" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A494" s="3">
+        <v>503803716</v>
+      </c>
+      <c r="B494" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="C494" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D494" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E494" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="495" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A495" s="3">
+        <v>503803715</v>
+      </c>
+      <c r="B495" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="C495" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D495" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E495" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="496" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A496" s="3">
+        <v>503800354</v>
+      </c>
+      <c r="B496" s="3" t="s">
+        <v>766</v>
+      </c>
+      <c r="C496" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D496" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E496" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="497" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A497" s="3">
+        <v>503802360</v>
+      </c>
+      <c r="B497" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="C497" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D497" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E497" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="498" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A498" s="3">
+        <v>503801337</v>
+      </c>
+      <c r="B498" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="C498" s="5">
+        <v>2700</v>
+      </c>
+      <c r="D498" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E498" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="499" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A499" s="3">
+        <v>503797420</v>
+      </c>
+      <c r="B499" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="C499" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D499" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E499" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="500" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A500" s="3">
+        <v>503800356</v>
+      </c>
+      <c r="B500" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="C500" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D500" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E500" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="501" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A501" s="3">
+        <v>503794515</v>
+      </c>
+      <c r="B501" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="C501" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D501" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E501" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="502" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A502" s="3">
+        <v>503804541</v>
+      </c>
+      <c r="B502" s="3" t="s">
+        <v>800</v>
+      </c>
+      <c r="C502" s="5">
+        <v>1640</v>
+      </c>
+      <c r="D502" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E502" s="6">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="503" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A503" s="3">
+        <v>503806499</v>
+      </c>
+      <c r="B503" s="3" t="s">
+        <v>767</v>
+      </c>
+      <c r="C503" s="5">
+        <v>1600</v>
+      </c>
+      <c r="D503" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E503" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="504" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A504" s="3">
+        <v>503800794</v>
+      </c>
+      <c r="B504" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="C504" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D504" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E504" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="505" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A505" s="3">
+        <v>503801298</v>
+      </c>
+      <c r="B505" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="C505" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D505" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E505" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="506" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A506" s="3">
+        <v>503801291</v>
+      </c>
+      <c r="B506" s="3" t="s">
+        <v>770</v>
+      </c>
+      <c r="C506" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D506" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E506" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="507" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A507" s="3">
+        <v>503806494</v>
+      </c>
+      <c r="B507" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="C507" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D507" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E507" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="508" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A508" s="3">
+        <v>503797421</v>
+      </c>
+      <c r="B508" s="3" t="s">
+        <v>772</v>
+      </c>
+      <c r="C508" s="5">
+        <v>1800</v>
+      </c>
+      <c r="D508" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E508" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="509" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A509" s="3">
+        <v>503804544</v>
+      </c>
+      <c r="B509" s="3" t="s">
+        <v>801</v>
+      </c>
+      <c r="C509" s="5">
+        <v>1530</v>
+      </c>
+      <c r="D509" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E509" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="510" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A510" s="3">
+        <v>503806160</v>
+      </c>
+      <c r="B510" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="C510" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D510" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E510" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="511" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A511" s="3">
+        <v>503804540</v>
+      </c>
+      <c r="B511" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="C511" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D511" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E511" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="512" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A512" s="3">
+        <v>503806204</v>
+      </c>
+      <c r="B512" s="3" t="s">
+        <v>804</v>
+      </c>
+      <c r="C512" s="5">
+        <v>3000</v>
+      </c>
+      <c r="D512" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E512" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="513" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A513" s="3">
+        <v>503806473</v>
+      </c>
+      <c r="B513" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="C513" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D513" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E513" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="514" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A514" s="3">
+        <v>503806203</v>
+      </c>
+      <c r="B514" s="3" t="s">
+        <v>806</v>
+      </c>
+      <c r="C514" s="5">
+        <v>2200</v>
+      </c>
+      <c r="D514" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E514" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="515" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A515" s="3">
+        <v>503806205</v>
+      </c>
+      <c r="B515" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="C515" s="5">
+        <v>3000</v>
+      </c>
+      <c r="D515" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E515" s="6">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="516" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A516" s="3">
+        <v>503809558</v>
+      </c>
+      <c r="B516" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="C516" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D516" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E516" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="517" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A517" s="3">
+        <v>503809553</v>
+      </c>
+      <c r="B517" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="C517" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D517" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E517" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="518" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A518" s="3">
+        <v>503806500</v>
+      </c>
+      <c r="B518" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="C518" s="5">
+        <v>2700</v>
+      </c>
+      <c r="D518" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E518" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="519" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A519" s="3">
+        <v>503809105</v>
+      </c>
+      <c r="B519" s="3" t="s">
+        <v>776</v>
+      </c>
+      <c r="C519" s="5">
+        <v>1000</v>
+      </c>
+      <c r="D519" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E519" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="520" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A520" s="3">
+        <v>503809559</v>
+      </c>
+      <c r="B520" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="C520" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D520" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E520" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="521" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A521" s="3">
+        <v>503809555</v>
+      </c>
+      <c r="B521" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="C521" s="5">
+        <v>2100</v>
+      </c>
+      <c r="D521" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E521" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="522" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A522" s="3">
+        <v>503809554</v>
+      </c>
+      <c r="B522" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="C522" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D522" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E522" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="523" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A523" s="3">
+        <v>503806474</v>
+      </c>
+      <c r="B523" s="3" t="s">
+        <v>808</v>
+      </c>
+      <c r="C523" s="5">
+        <v>1400</v>
+      </c>
+      <c r="D523" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E523" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="524" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A524" s="3">
+        <v>503804474</v>
+      </c>
+      <c r="B524" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="C524" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D524" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E524" s="6">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="525" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A525" s="3">
+        <v>503809560</v>
+      </c>
+      <c r="B525" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="C525" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D525" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E525" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="526" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A526" s="3">
+        <v>503809557</v>
+      </c>
+      <c r="B526" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="C526" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D526" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E526" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="527" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A527" s="3">
+        <v>503812294</v>
+      </c>
+      <c r="B527" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="C527" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D527" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E527" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="528" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A528" s="3">
+        <v>503812171</v>
+      </c>
+      <c r="B528" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="C528" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D528" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E528" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="529" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A529" s="3">
+        <v>503812173</v>
+      </c>
+      <c r="B529" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="C529" s="5">
+        <v>1000</v>
+      </c>
+      <c r="D529" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E529" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="530" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A530" s="3">
+        <v>503812172</v>
+      </c>
+      <c r="B530" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="C530" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D530" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E530" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="531" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A531" s="3">
+        <v>503812151</v>
+      </c>
+      <c r="B531" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="C531" s="5">
+        <v>1300</v>
+      </c>
+      <c r="D531" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E531" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="532" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A532" s="3">
+        <v>503813541</v>
+      </c>
+      <c r="B532" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="C532" s="5">
+        <v>2700</v>
+      </c>
+      <c r="D532" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E532" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="533" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A533" s="3">
+        <v>503812174</v>
+      </c>
+      <c r="B533" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="C533" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D533" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E533" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="534" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A534" s="3">
+        <v>503780330</v>
+      </c>
+      <c r="B534" s="3" t="s">
+        <v>789</v>
+      </c>
+      <c r="C534" s="5">
+        <v>1400</v>
+      </c>
+      <c r="D534" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E534" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="535" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A535" s="3">
+        <v>503812169</v>
+      </c>
+      <c r="B535" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="C535" s="5">
+        <v>2100</v>
+      </c>
+      <c r="D535" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E535" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="536" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A536" s="3">
+        <v>503812170</v>
+      </c>
+      <c r="B536" s="3" t="s">
+        <v>791</v>
+      </c>
+      <c r="C536" s="5">
+        <v>2200</v>
+      </c>
+      <c r="D536" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E536" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="537" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A537" s="3">
+        <v>503812175</v>
+      </c>
+      <c r="B537" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C537" s="5">
+        <v>1000</v>
+      </c>
+      <c r="D537" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E537" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="538" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A538" s="3">
+        <v>503804497</v>
+      </c>
+      <c r="B538" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="C538" s="5">
+        <v>1900</v>
+      </c>
+      <c r="D538" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E538" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="539" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A539" s="3">
+        <v>503812164</v>
+      </c>
+      <c r="B539" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="C539" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D539" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E539" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="540" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A540" s="3">
+        <v>503804498</v>
+      </c>
+      <c r="B540" s="3" t="s">
+        <v>812</v>
+      </c>
+      <c r="C540" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D540" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E540" s="6">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="541" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A541" s="3">
+        <v>503806491</v>
+      </c>
+      <c r="B541" s="3" t="s">
+        <v>793</v>
+      </c>
+      <c r="C541" s="5">
+        <v>1800</v>
+      </c>
+      <c r="D541" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E541" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="542" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A542" s="3">
+        <v>503814546</v>
+      </c>
+      <c r="B542" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="C542" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D542" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E542" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="543" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A543" s="3">
+        <v>503812143</v>
+      </c>
+      <c r="B543" s="3" t="s">
+        <v>813</v>
+      </c>
+      <c r="C543" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D543" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E543" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="544" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A544" s="3">
+        <v>503809077</v>
+      </c>
+      <c r="B544" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="C544" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D544" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E544" s="6">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="545" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A545" s="3">
+        <v>503812146</v>
+      </c>
+      <c r="B545" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="C545" s="5">
+        <v>1000</v>
+      </c>
+      <c r="D545" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E545" s="6">
+        <v>46164</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F490" xr:uid="{4D5B24D8-C2AF-482A-9CC6-491ED0721327}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F490">
-      <sortCondition ref="E1:E233"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F545">
+      <sortCondition ref="E1:E490"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
데이터 업데이트 2026-06-01 (벌크 6701개, MAE 11.97%)
</commit_message>
<xml_diff>
--- a/data/disposal.xlsx
+++ b/data/disposal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cosmaxdt-my.sharepoint.com/personal/djlee_cosmax_com/Documents/바탕 화면/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="8_{130E5389-1375-4C82-BE1D-2D037779CF4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A81B6BFD-70B9-4E0E-9C9D-D23061C84D92}"/>
+  <xr:revisionPtr revIDLastSave="141" documentId="8_{130E5389-1375-4C82-BE1D-2D037779CF4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A2BD4D4-ED8F-4904-8A83-6446C23C5BE9}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{156CA689-9E30-4938-99C3-2C7A464D90AA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1885" uniqueCount="909">
   <si>
     <t>생산오더</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -3128,6 +3128,174 @@
   </si>
   <si>
     <t>3MEM00567160</t>
+  </si>
+  <si>
+    <t>3CLO13187140</t>
+  </si>
+  <si>
+    <t>3CLO13187110</t>
+  </si>
+  <si>
+    <t>3CLO13982140</t>
+  </si>
+  <si>
+    <t>3CLO13982155</t>
+  </si>
+  <si>
+    <t>3CLO13009150</t>
+  </si>
+  <si>
+    <t>3IWD00330120</t>
+  </si>
+  <si>
+    <t>3CLO13009200</t>
+  </si>
+  <si>
+    <t>3CLO13009140</t>
+  </si>
+  <si>
+    <t>3CLO13010110</t>
+  </si>
+  <si>
+    <t>3IWD00328170</t>
+  </si>
+  <si>
+    <t>3CLO13010200</t>
+  </si>
+  <si>
+    <t>3MEM08566130</t>
+  </si>
+  <si>
+    <t>3OLV10265230</t>
+  </si>
+  <si>
+    <t>3IAN10193140</t>
+  </si>
+  <si>
+    <t>3IWD00113310</t>
+  </si>
+  <si>
+    <t>3CLO13982115</t>
+  </si>
+  <si>
+    <t>3CLO13187120</t>
+  </si>
+  <si>
+    <t>3IAN10213110</t>
+  </si>
+  <si>
+    <t>3CLO13009210</t>
+  </si>
+  <si>
+    <t>3IAN10126140</t>
+  </si>
+  <si>
+    <t>3IWD00342150</t>
+  </si>
+  <si>
+    <t>3IAN10126120</t>
+  </si>
+  <si>
+    <t>3OLV11112115</t>
+  </si>
+  <si>
+    <t>3DZK00347180</t>
+  </si>
+  <si>
+    <t>3MEM00824121</t>
+  </si>
+  <si>
+    <t>3MEM08540110</t>
+  </si>
+  <si>
+    <t>3IAN10193120</t>
+  </si>
+  <si>
+    <t>3IAN10378160</t>
+  </si>
+  <si>
+    <t>3IAN10301120</t>
+  </si>
+  <si>
+    <t>3MEM00678132</t>
+  </si>
+  <si>
+    <t>3CLO13233180</t>
+  </si>
+  <si>
+    <t>3CLO13233170</t>
+  </si>
+  <si>
+    <t>3CLO13233160</t>
+  </si>
+  <si>
+    <t>3MEM00567150</t>
+  </si>
+  <si>
+    <t>3ENP00739160</t>
+  </si>
+  <si>
+    <t>3ENP00739153</t>
+  </si>
+  <si>
+    <t>3ENP00739152</t>
+  </si>
+  <si>
+    <t>3ENP00739151</t>
+  </si>
+  <si>
+    <t>3NRP01710140</t>
+  </si>
+  <si>
+    <t>3ENP00739120</t>
+  </si>
+  <si>
+    <t>3ENP00739180</t>
+  </si>
+  <si>
+    <t>3CLO13971150</t>
+  </si>
+  <si>
+    <t>3NRP01577210</t>
+  </si>
+  <si>
+    <t>3ENP00739140</t>
+  </si>
+  <si>
+    <t>3ENP00739130</t>
+  </si>
+  <si>
+    <t>3AML00049111</t>
+  </si>
+  <si>
+    <t>3AML00107112</t>
+  </si>
+  <si>
+    <t>3ENP00739270</t>
+  </si>
+  <si>
+    <t>3AML00059111</t>
+  </si>
+  <si>
+    <t>3NDA01166111</t>
+  </si>
+  <si>
+    <t>3ENP00739190</t>
+  </si>
+  <si>
+    <t>3NDA01166131</t>
+  </si>
+  <si>
+    <t>3NDA01166121</t>
+  </si>
+  <si>
+    <t>3IWD00478110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3NDA01166141	</t>
+  </si>
+  <si>
+    <t>3AML00048112</t>
   </si>
 </sst>
 </file>
@@ -3583,7 +3751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D5B24D8-C2AF-482A-9CC6-491ED0721327}">
-  <dimension ref="A1:F329"/>
+  <dimension ref="A1:F356"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" style="3" bestFit="1" customWidth="1"/>
@@ -9190,9 +9358,468 @@
         <v>46164</v>
       </c>
     </row>
+    <row r="330" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A330" s="3">
+        <v>503814366</v>
+      </c>
+      <c r="B330" s="3" t="s">
+        <v>882</v>
+      </c>
+      <c r="C330" s="5">
+        <v>500</v>
+      </c>
+      <c r="D330" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E330" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="331" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A331" s="3">
+        <v>503812090</v>
+      </c>
+      <c r="B331" s="3" t="s">
+        <v>883</v>
+      </c>
+      <c r="C331" s="5">
+        <v>500</v>
+      </c>
+      <c r="D331" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E331" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="332" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A332" s="3">
+        <v>503812090</v>
+      </c>
+      <c r="B332" s="3" t="s">
+        <v>884</v>
+      </c>
+      <c r="C332" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D332" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E332" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="333" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A333" s="3">
+        <v>503812090</v>
+      </c>
+      <c r="B333" s="3" t="s">
+        <v>885</v>
+      </c>
+      <c r="C333" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D333" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E333" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="334" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A334" s="3">
+        <v>503812038</v>
+      </c>
+      <c r="B334" s="3" t="s">
+        <v>886</v>
+      </c>
+      <c r="C334" s="5">
+        <v>500</v>
+      </c>
+      <c r="D334" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E334" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="335" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A335" s="3">
+        <v>503819428</v>
+      </c>
+      <c r="B335" s="3" t="s">
+        <v>887</v>
+      </c>
+      <c r="C335" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D335" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E335" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="336" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A336" s="3">
+        <v>503827186</v>
+      </c>
+      <c r="B336" s="3" t="s">
+        <v>888</v>
+      </c>
+      <c r="C336" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D336" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E336" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="337" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A337" s="3">
+        <v>503827186</v>
+      </c>
+      <c r="B337" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="C337" s="5">
+        <v>100</v>
+      </c>
+      <c r="D337" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E337" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="338" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A338" s="3">
+        <v>503827186</v>
+      </c>
+      <c r="B338" s="3" t="s">
+        <v>890</v>
+      </c>
+      <c r="C338" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D338" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E338" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="339" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A339" s="3">
+        <v>503816513</v>
+      </c>
+      <c r="B339" s="3" t="s">
+        <v>891</v>
+      </c>
+      <c r="C339" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D339" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E339" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="340" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A340" s="3">
+        <v>503819427</v>
+      </c>
+      <c r="B340" s="3" t="s">
+        <v>892</v>
+      </c>
+      <c r="C340" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D340" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E340" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="341" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A341" s="3">
+        <v>503819430</v>
+      </c>
+      <c r="B341" s="3" t="s">
+        <v>893</v>
+      </c>
+      <c r="C341" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D341" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E341" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="342" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A342" s="3">
+        <v>503818413</v>
+      </c>
+      <c r="B342" s="3" t="s">
+        <v>894</v>
+      </c>
+      <c r="C342" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D342" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E342" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="343" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A343" s="3">
+        <v>503806531</v>
+      </c>
+      <c r="B343" s="3" t="s">
+        <v>895</v>
+      </c>
+      <c r="C343" s="5">
+        <v>2600</v>
+      </c>
+      <c r="D343" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E343" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="344" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A344" s="3">
+        <v>503816803</v>
+      </c>
+      <c r="B344" s="3" t="s">
+        <v>896</v>
+      </c>
+      <c r="C344" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D344" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E344" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="345" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A345" s="3">
+        <v>503816682</v>
+      </c>
+      <c r="B345" s="3" t="s">
+        <v>897</v>
+      </c>
+      <c r="C345" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D345" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E345" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="346" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A346" s="3">
+        <v>503812087</v>
+      </c>
+      <c r="B346" s="3" t="s">
+        <v>898</v>
+      </c>
+      <c r="C346" s="5">
+        <v>500</v>
+      </c>
+      <c r="D346" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E346" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="347" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A347" s="3">
+        <v>503812089</v>
+      </c>
+      <c r="B347" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="C347" s="5">
+        <v>1000</v>
+      </c>
+      <c r="D347" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E347" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="348" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A348" s="3">
+        <v>503819429</v>
+      </c>
+      <c r="B348" s="3" t="s">
+        <v>900</v>
+      </c>
+      <c r="C348" s="5">
+        <v>2600</v>
+      </c>
+      <c r="D348" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E348" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="349" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A349" s="3">
+        <v>503812088</v>
+      </c>
+      <c r="B349" s="3" t="s">
+        <v>901</v>
+      </c>
+      <c r="C349" s="5">
+        <v>1800</v>
+      </c>
+      <c r="D349" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E349" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="350" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A350" s="3">
+        <v>503819432</v>
+      </c>
+      <c r="B350" s="3" t="s">
+        <v>902</v>
+      </c>
+      <c r="C350" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D350" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E350" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="351" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A351" s="3">
+        <v>503819431</v>
+      </c>
+      <c r="B351" s="3" t="s">
+        <v>903</v>
+      </c>
+      <c r="C351" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D351" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E351" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="352" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A352" s="3">
+        <v>503819434</v>
+      </c>
+      <c r="B352" s="3" t="s">
+        <v>904</v>
+      </c>
+      <c r="C352" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D352" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E352" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="353" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A353" s="3">
+        <v>503819433</v>
+      </c>
+      <c r="B353" s="3" t="s">
+        <v>905</v>
+      </c>
+      <c r="C353" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D353" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E353" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="354" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A354" s="3">
+        <v>503808976</v>
+      </c>
+      <c r="B354" s="3" t="s">
+        <v>906</v>
+      </c>
+      <c r="C354" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D354" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E354" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="355" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A355" s="3">
+        <v>503819435</v>
+      </c>
+      <c r="B355" s="3" t="s">
+        <v>907</v>
+      </c>
+      <c r="C355" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D355" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E355" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="356" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A356" s="3">
+        <v>503816681</v>
+      </c>
+      <c r="B356" s="3" t="s">
+        <v>908</v>
+      </c>
+      <c r="C356" s="5">
+        <v>1000</v>
+      </c>
+      <c r="D356" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E356" s="6">
+        <v>46171</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F290" xr:uid="{4D5B24D8-C2AF-482A-9CC6-491ED0721327}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F329">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F356">
       <sortCondition ref="E1:E290"/>
     </sortState>
   </autoFilter>
@@ -9203,7 +9830,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2F62A61-38E3-43AD-974B-FDA325720BCC}">
-  <dimension ref="A1:F545"/>
+  <dimension ref="A1:F582"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" style="3" bestFit="1" customWidth="1"/>
@@ -18486,9 +19113,638 @@
         <v>46164</v>
       </c>
     </row>
+    <row r="546" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A546" s="3">
+        <v>503814455</v>
+      </c>
+      <c r="B546" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="C546" s="5">
+        <v>2600</v>
+      </c>
+      <c r="D546" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E546" s="6">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="547" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A547" s="3">
+        <v>503814454</v>
+      </c>
+      <c r="B547" s="3" t="s">
+        <v>854</v>
+      </c>
+      <c r="C547" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D547" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E547" s="6">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="548" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A548" s="3">
+        <v>503812292</v>
+      </c>
+      <c r="B548" s="3" t="s">
+        <v>855</v>
+      </c>
+      <c r="C548" s="5">
+        <v>1800</v>
+      </c>
+      <c r="D548" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E548" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="549" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A549" s="3">
+        <v>503817171</v>
+      </c>
+      <c r="B549" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="C549" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D549" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E549" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="550" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A550" s="3">
+        <v>503812293</v>
+      </c>
+      <c r="B550" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="C550" s="5">
+        <v>1700</v>
+      </c>
+      <c r="D550" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E550" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="551" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A551" s="3">
+        <v>503812153</v>
+      </c>
+      <c r="B551" s="3" t="s">
+        <v>857</v>
+      </c>
+      <c r="C551" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D551" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E551" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="552" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A552" s="3">
+        <v>503817182</v>
+      </c>
+      <c r="B552" s="3" t="s">
+        <v>858</v>
+      </c>
+      <c r="C552" s="5">
+        <v>2900</v>
+      </c>
+      <c r="D552" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E552" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="553" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A553" s="3">
+        <v>503812157</v>
+      </c>
+      <c r="B553" s="3" t="s">
+        <v>859</v>
+      </c>
+      <c r="C553" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D553" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E553" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="554" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A554" s="3">
+        <v>503809618</v>
+      </c>
+      <c r="B554" s="3" t="s">
+        <v>868</v>
+      </c>
+      <c r="C554" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D554" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E554" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="555" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A555" s="3">
+        <v>503814459</v>
+      </c>
+      <c r="B555" s="3" t="s">
+        <v>869</v>
+      </c>
+      <c r="C555" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D555" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E555" s="6">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="556" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A556" s="3">
+        <v>503817177</v>
+      </c>
+      <c r="B556" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="C556" s="5">
+        <v>1600</v>
+      </c>
+      <c r="D556" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E556" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="557" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A557" s="3">
+        <v>503812152</v>
+      </c>
+      <c r="B557" s="3" t="s">
+        <v>860</v>
+      </c>
+      <c r="C557" s="5">
+        <v>2300</v>
+      </c>
+      <c r="D557" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E557" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="558" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A558" s="3">
+        <v>503817174</v>
+      </c>
+      <c r="B558" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="C558" s="5">
+        <v>1400</v>
+      </c>
+      <c r="D558" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E558" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="559" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A559" s="3">
+        <v>503821903</v>
+      </c>
+      <c r="B559" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="C559" s="5">
+        <v>1400</v>
+      </c>
+      <c r="D559" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E559" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="560" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A560" s="3">
+        <v>503771350</v>
+      </c>
+      <c r="B560" s="3" t="s">
+        <v>870</v>
+      </c>
+      <c r="C560" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D560" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E560" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="561" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A561" s="3">
+        <v>503809893</v>
+      </c>
+      <c r="B561" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="C561" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D561" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E561" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="562" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A562" s="3">
+        <v>503817189</v>
+      </c>
+      <c r="B562" s="3" t="s">
+        <v>872</v>
+      </c>
+      <c r="C562" s="5">
+        <v>2700</v>
+      </c>
+      <c r="D562" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E562" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="563" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A563" s="3">
+        <v>503820952</v>
+      </c>
+      <c r="B563" s="3" t="s">
+        <v>873</v>
+      </c>
+      <c r="C563" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D563" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E563" s="6">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="564" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A564" s="3">
+        <v>503819091</v>
+      </c>
+      <c r="B564" s="3" t="s">
+        <v>861</v>
+      </c>
+      <c r="C564" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D564" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E564" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="565" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A565" s="3">
+        <v>503819135</v>
+      </c>
+      <c r="B565" s="3" t="s">
+        <v>862</v>
+      </c>
+      <c r="C565" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D565" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E565" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="566" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A566" s="3">
+        <v>503819100</v>
+      </c>
+      <c r="B566" s="3" t="s">
+        <v>863</v>
+      </c>
+      <c r="C566" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D566" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E566" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="567" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A567" s="3">
+        <v>503821769</v>
+      </c>
+      <c r="B567" s="3" t="s">
+        <v>864</v>
+      </c>
+      <c r="C567" s="5">
+        <v>1900</v>
+      </c>
+      <c r="D567" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E567" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="568" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A568" s="3">
+        <v>503817187</v>
+      </c>
+      <c r="B568" s="3" t="s">
+        <v>874</v>
+      </c>
+      <c r="C568" s="5">
+        <v>3000</v>
+      </c>
+      <c r="D568" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E568" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="569" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A569" s="3">
+        <v>503826670</v>
+      </c>
+      <c r="B569" s="3" t="s">
+        <v>875</v>
+      </c>
+      <c r="C569" s="5">
+        <v>1900</v>
+      </c>
+      <c r="D569" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E569" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="570" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A570" s="3">
+        <v>503817169</v>
+      </c>
+      <c r="B570" s="3" t="s">
+        <v>876</v>
+      </c>
+      <c r="C570" s="5">
+        <v>3000</v>
+      </c>
+      <c r="D570" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E570" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="571" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A571" s="3">
+        <v>503817200</v>
+      </c>
+      <c r="B571" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="C571" s="5">
+        <v>1800</v>
+      </c>
+      <c r="D571" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E571" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="572" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A572" s="3">
+        <v>503817201</v>
+      </c>
+      <c r="B572" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="C572" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D572" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E572" s="6">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="573" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A573" s="3">
+        <v>503821881</v>
+      </c>
+      <c r="B573" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="C573" s="5">
+        <v>1900</v>
+      </c>
+      <c r="D573" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E573" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="574" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A574" s="3">
+        <v>503821915</v>
+      </c>
+      <c r="B574" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="C574" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D574" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E574" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="575" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A575" s="3">
+        <v>503826262</v>
+      </c>
+      <c r="B575" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="C575" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D575" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E575" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="576" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A576" s="3">
+        <v>503827603</v>
+      </c>
+      <c r="B576" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="C576" s="5">
+        <v>2700</v>
+      </c>
+      <c r="D576" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E576" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="577" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A577" s="3">
+        <v>503821870</v>
+      </c>
+      <c r="B577" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="C577" s="5">
+        <v>1800</v>
+      </c>
+      <c r="D577" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E577" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="578" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A578" s="3">
+        <v>503826260</v>
+      </c>
+      <c r="B578" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="C578" s="5">
+        <v>2700</v>
+      </c>
+      <c r="D578" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E578" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="579" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A579" s="3">
+        <v>503826578</v>
+      </c>
+      <c r="B579" s="3" t="s">
+        <v>880</v>
+      </c>
+      <c r="C579" s="5">
+        <v>2600</v>
+      </c>
+      <c r="D579" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E579" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="580" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A580" s="3">
+        <v>503826578</v>
+      </c>
+      <c r="B580" s="3" t="s">
+        <v>880</v>
+      </c>
+      <c r="C580" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D580" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E580" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="581" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A581" s="3">
+        <v>503826444</v>
+      </c>
+      <c r="B581" s="3" t="s">
+        <v>881</v>
+      </c>
+      <c r="C581" s="5">
+        <v>2500</v>
+      </c>
+      <c r="D581" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E581" s="6">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="582" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A582" s="3">
+        <v>503821927</v>
+      </c>
+      <c r="B582" s="3" t="s">
+        <v>677</v>
+      </c>
+      <c r="C582" s="5">
+        <v>1000</v>
+      </c>
+      <c r="D582" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E582" s="6">
+        <v>46171</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F490" xr:uid="{4D5B24D8-C2AF-482A-9CC6-491ED0721327}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F545">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F582">
       <sortCondition ref="E1:E490"/>
     </sortState>
   </autoFilter>

</xml_diff>